<commit_message>
Temporary excel files filtered, unique early applicants count added
</commit_message>
<xml_diff>
--- a/templates/programs.xlsx
+++ b/templates/programs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tijuanap\Programs\HSE_dashboard\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34D599A2-8AF8-458B-B3ED-2FCD7DAE8733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3AC7C3-228B-4E9B-B657-0846FDC5A672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{B52EB287-D043-DE4C-B969-F80F8215C3F0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{B52EB287-D043-DE4C-B969-F80F8215C3F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,21 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$48</definedName>
   </definedNames>
-  <calcPr calcId="179021" refMode="R1C1"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -201,9 +212,6 @@
     <t>Прикладная лингвистика: обучение иностранному языку и перевод в цифровой среде</t>
   </si>
   <si>
-    <t>ПРИКЛИНГ.Прикладная лингвистика обучение иностранному языку и перевод в цифровой среде / НИУ ВШЭ СанктПетербург / 450403 Фундаментальная и прикладная лингвистика / Факультет СанктПетербургская школа гуманитарных наук и искусств / Магистратура</t>
-  </si>
-  <si>
     <t>Прикладная социальная психология</t>
   </si>
   <si>
@@ -370,6 +378,9 @@
   </si>
   <si>
     <t>start_year</t>
+  </si>
+  <si>
+    <t>ПРИКЛИНГ. Прикладная лингвистика обучение иностранному языку и перевод в цифровой среде / НИУ ВШЭ СанктПетербург / 450403 Фундаментальная и прикладная лингвистика / Факультет СанктПетербургская школа гуманитарных наук и искусств / Магистратура</t>
   </si>
 </sst>
 </file>
@@ -811,13 +822,13 @@
         <v>8</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="K1" s="5" t="s">
-        <v>107</v>
-      </c>
       <c r="L1" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -852,7 +863,7 @@
         <v>-4147228289</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L2" s="2">
         <v>2024</v>
@@ -890,7 +901,7 @@
         <v>-972833656</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L3" s="2">
         <v>2021</v>
@@ -898,7 +909,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>10</v>
@@ -920,10 +931,10 @@
         <v>50</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L4" s="2">
         <v>2026</v>
@@ -966,7 +977,7 @@
         <v>-4749312259</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L5" s="2">
         <v>2025</v>
@@ -1009,7 +1020,7 @@
         <v>-4046984274</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L6" s="2">
         <v>2024</v>
@@ -1081,7 +1092,7 @@
         <v>-4139485502</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L8" s="2">
         <v>2021</v>
@@ -1119,7 +1130,7 @@
         <v>-1002100789923</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L9" s="2">
         <v>2023</v>
@@ -1157,7 +1168,7 @@
         <v>-1001998842044</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L10" s="2">
         <v>2024</v>
@@ -1195,7 +1206,7 @@
         <v>-4171683633</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L11" s="2">
         <v>2024</v>
@@ -1203,7 +1214,7 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>10</v>
@@ -1224,13 +1235,13 @@
         <v>100</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J12" s="5">
         <v>-4867774341</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L12" s="2">
         <v>2026</v>
@@ -1268,7 +1279,7 @@
         <v>-613642779</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L13" s="2">
         <v>2021</v>
@@ -1306,7 +1317,7 @@
         <v>-4198260355</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L14" s="2">
         <v>2024</v>
@@ -1344,7 +1355,7 @@
         <v>-688995997</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L15" s="2">
         <v>2021</v>
@@ -1382,7 +1393,7 @@
         <v>-1002192951552</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L16" s="2">
         <v>2024</v>
@@ -1420,7 +1431,7 @@
         <v>-5240425567</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L17" s="2">
         <v>2022</v>
@@ -1458,7 +1469,7 @@
         <v>-1002670463110</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L18" s="2">
         <v>2025</v>
@@ -1496,7 +1507,7 @@
         <v>-772593583</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L19" s="2">
         <v>2021</v>
@@ -1534,7 +1545,7 @@
         <v>-5203561930</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L20" s="2">
         <v>2022</v>
@@ -1572,7 +1583,7 @@
         <v>-5028978394</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L21" s="2">
         <v>2021</v>
@@ -1580,7 +1591,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>10</v>
@@ -1604,13 +1615,13 @@
         <v>100</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J22" s="5">
         <v>-1002216681454</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L22" s="2">
         <v>2020</v>
@@ -1648,7 +1659,7 @@
         <v>-4186647978</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L23" s="2">
         <v>2021</v>
@@ -1686,7 +1697,7 @@
         <v>-1002500028103</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L24" s="2">
         <v>2024</v>
@@ -1724,7 +1735,7 @@
         <v>-1002508354725</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L25" s="2">
         <v>2025</v>
@@ -1756,13 +1767,13 @@
         <v>100</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>56</v>
+        <v>112</v>
       </c>
       <c r="J26" s="5">
         <v>-1002562197059</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L26" s="2">
         <v>2025</v>
@@ -1770,7 +1781,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>10</v>
@@ -1794,13 +1805,13 @@
         <v>100</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J27" s="5">
         <v>-878424227</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L27" s="2">
         <v>2022</v>
@@ -1808,7 +1819,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>19</v>
@@ -1832,13 +1843,13 @@
         <v>50</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J28" s="5">
         <v>-4709453212</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L28" s="2">
         <v>2024</v>
@@ -1846,7 +1857,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>10</v>
@@ -1867,13 +1878,13 @@
         <v>100</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J29" s="5">
         <v>-4906367157</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L29" s="2">
         <v>2026</v>
@@ -1881,7 +1892,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>10</v>
@@ -1905,13 +1916,13 @@
         <v>100</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J30" s="5">
         <v>-942218135</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L30" s="2">
         <v>2023</v>
@@ -1919,7 +1930,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>10</v>
@@ -1943,13 +1954,13 @@
         <v>100</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J31" s="5">
         <v>-4073830216</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L31" s="2">
         <v>2024</v>
@@ -1957,7 +1968,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>10</v>
@@ -1981,13 +1992,13 @@
         <v>100</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J32" s="13">
         <v>-1002573664656</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L32" s="2">
         <v>2024</v>
@@ -1995,7 +2006,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>10</v>
@@ -2016,13 +2027,13 @@
         <v>100</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J33" s="5">
         <v>-5079133035</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L33" s="2">
         <v>2026</v>
@@ -2030,7 +2041,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>19</v>
@@ -2054,13 +2065,13 @@
         <v>100</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J34" s="5">
         <v>-4542263709</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L34" s="2">
         <v>2025</v>
@@ -2068,7 +2079,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>10</v>
@@ -2092,13 +2103,13 @@
         <v>100</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J35" s="5">
         <v>-4102964588</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L35" s="2">
         <v>2024</v>
@@ -2106,7 +2117,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>10</v>
@@ -2130,13 +2141,13 @@
         <v>100</v>
       </c>
       <c r="I36" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J36" s="5">
         <v>-4092316930</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L36" s="2">
         <v>2024</v>
@@ -2144,7 +2155,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>10</v>
@@ -2165,13 +2176,13 @@
         <v>100</v>
       </c>
       <c r="I37" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J37" s="5">
         <v>-4891752359</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L37" s="2">
         <v>2026</v>
@@ -2179,7 +2190,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>10</v>
@@ -2203,13 +2214,13 @@
         <v>100</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J38" s="5">
         <v>-892164059</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L38" s="2">
         <v>2023</v>
@@ -2217,7 +2228,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>10</v>
@@ -2241,13 +2252,13 @@
         <v>100</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J39" s="5">
         <v>-1002035879507</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L39" s="2">
         <v>2022</v>
@@ -2255,7 +2266,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>19</v>
@@ -2281,7 +2292,7 @@
         <v>-4980553625</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L40" s="2">
         <v>2026</v>
@@ -2289,7 +2300,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>10</v>
@@ -2311,13 +2322,13 @@
         <v>100</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J41" s="5">
         <v>-4875829621</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L41" s="2">
         <v>2026</v>
@@ -2325,7 +2336,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>10</v>
@@ -2349,13 +2360,13 @@
         <v>100</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J42" s="5">
         <v>-1002070587931</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L42" s="2">
         <v>2021</v>
@@ -2363,7 +2374,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>10</v>
@@ -2387,13 +2398,13 @@
         <v>100</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J43" s="5">
         <v>-889355707</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L43" s="2">
         <v>2021</v>
@@ -2401,7 +2412,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>10</v>
@@ -2425,13 +2436,13 @@
         <v>100</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J44" s="5">
         <v>-4602706028</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L44" s="2">
         <v>2025</v>
@@ -2439,7 +2450,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>10</v>
@@ -2463,13 +2474,13 @@
         <v>100</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J45" s="5">
         <v>-824212567</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L45" s="2">
         <v>2023</v>
@@ -2477,7 +2488,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>10</v>
@@ -2501,13 +2512,13 @@
         <v>100</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J46" s="5">
         <v>-4595042190</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L46" s="2">
         <v>2025</v>
@@ -2515,7 +2526,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>10</v>
@@ -2539,13 +2550,13 @@
         <v>100</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J47" s="5">
         <v>-1002012887954</v>
       </c>
       <c r="K47" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L47" s="2">
         <v>2021</v>
@@ -2553,7 +2564,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>19</v>
@@ -2577,13 +2588,13 @@
         <v>100</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J48" s="5">
         <v>-4997646337</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L48" s="2">
         <v>2022</v>

</xml_diff>

<commit_message>
Minor fixes: wrong birthdays @ early invitation, int.design alias
</commit_message>
<xml_diff>
--- a/templates/programs.xlsx
+++ b/templates/programs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tijuanap\Programs\HSE_dashboard\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7F687C-FFC9-43E3-BCA7-37398801C80E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374D700-AEC6-4FF4-B9AF-EE4DD24D9C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{B52EB287-D043-DE4C-B969-F80F8215C3F0}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$48</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -158,9 +158,6 @@
     <t>Интерактивный дизайн</t>
   </si>
   <si>
-    <t>ИНТДИЗ. Интерактивный дизайн / Москва / 540401 Дизайн / факультет креативных индустрий / Магистратура</t>
-  </si>
-  <si>
     <t>Искусственный интеллект</t>
   </si>
   <si>
@@ -408,6 +405,9 @@
   </si>
   <si>
     <t>УТИН. Управление технологическими инновациями</t>
+  </si>
+  <si>
+    <t>ИНТДИЗ. Интерактивный дизайн</t>
   </si>
 </sst>
 </file>
@@ -798,7 +798,8 @@
   <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="9" width="11.25" style="3"/>
+    <col min="2" max="8" width="11.25" style="3"/>
+    <col min="9" max="9" width="42.875" style="3" customWidth="1"/>
     <col min="10" max="10" width="15.875" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.75" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.25" style="3"/>
@@ -834,13 +835,13 @@
         <v>8</v>
       </c>
       <c r="J1" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="K1" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="K1" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="L1" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -875,7 +876,7 @@
         <v>-4147228289</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L2" s="3">
         <v>2024</v>
@@ -913,7 +914,7 @@
         <v>-972833656</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L3" s="3">
         <v>2021</v>
@@ -921,7 +922,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>10</v>
@@ -945,10 +946,10 @@
         <v>50</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L4" s="3">
         <v>2026</v>
@@ -967,7 +968,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="3">
-        <v>700</v>
+        <v>560</v>
       </c>
       <c r="D5" s="4">
         <v>15</v>
@@ -991,7 +992,7 @@
         <v>-4749312259</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L5" s="3">
         <v>2025</v>
@@ -1034,7 +1035,7 @@
         <v>-4046984274</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L6" s="3">
         <v>2024</v>
@@ -1106,7 +1107,7 @@
         <v>-4139485502</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L8" s="3">
         <v>2021</v>
@@ -1144,7 +1145,7 @@
         <v>-1002100789923</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L9" s="3">
         <v>2023</v>
@@ -1182,7 +1183,7 @@
         <v>-1001998842044</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L10" s="3">
         <v>2024</v>
@@ -1214,13 +1215,13 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>30</v>
+        <v>113</v>
       </c>
       <c r="J11" s="6">
         <v>-4171683633</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L11" s="3">
         <v>2024</v>
@@ -1228,7 +1229,7 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>10</v>
@@ -1249,13 +1250,13 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J12" s="6">
         <v>-4867774341</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L12" s="3">
         <v>2026</v>
@@ -1263,7 +1264,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>10</v>
@@ -1287,13 +1288,13 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J13" s="6">
         <v>-613642779</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L13" s="3">
         <v>2021</v>
@@ -1301,7 +1302,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>10</v>
@@ -1325,13 +1326,13 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J14" s="6">
         <v>-4198260355</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L14" s="3">
         <v>2024</v>
@@ -1339,7 +1340,7 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>10</v>
@@ -1363,13 +1364,13 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J15" s="6">
         <v>-688995997</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L15" s="3">
         <v>2021</v>
@@ -1377,7 +1378,7 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>10</v>
@@ -1401,13 +1402,13 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J16" s="6">
         <v>-1002192951552</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L16" s="3">
         <v>2024</v>
@@ -1415,7 +1416,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>10</v>
@@ -1439,13 +1440,13 @@
         <v>50</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J17" s="6">
         <v>-5240425567</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L17" s="3">
         <v>2022</v>
@@ -1453,7 +1454,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>10</v>
@@ -1477,13 +1478,13 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J18" s="6">
         <v>-1002670463110</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L18" s="3">
         <v>2025</v>
@@ -1491,7 +1492,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>19</v>
@@ -1515,13 +1516,13 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J19" s="6">
         <v>-772593583</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L19" s="3">
         <v>2021</v>
@@ -1529,7 +1530,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>10</v>
@@ -1553,13 +1554,13 @@
         <v>50</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J20" s="6">
         <v>-5203561930</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L20" s="3">
         <v>2022</v>
@@ -1567,7 +1568,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>10</v>
@@ -1591,13 +1592,13 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J21" s="6">
         <v>-5028978394</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L21" s="3">
         <v>2021</v>
@@ -1605,7 +1606,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>10</v>
@@ -1629,13 +1630,13 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J22" s="6">
         <v>-1002216681454</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L22" s="3">
         <v>2020</v>
@@ -1643,7 +1644,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>10</v>
@@ -1667,13 +1668,13 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J23" s="6">
         <v>-4186647978</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L23" s="3">
         <v>2021</v>
@@ -1681,7 +1682,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>10</v>
@@ -1705,13 +1706,13 @@
         <v>100</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J24" s="6">
         <v>-1002500028103</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L24" s="3">
         <v>2024</v>
@@ -1719,7 +1720,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>10</v>
@@ -1743,13 +1744,13 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J25" s="6">
         <v>-1002508354725</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L25" s="3">
         <v>2025</v>
@@ -1757,7 +1758,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>10</v>
@@ -1781,13 +1782,13 @@
         <v>100</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J26" s="6">
         <v>-1002562197059</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L26" s="3">
         <v>2025</v>
@@ -1795,7 +1796,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>10</v>
@@ -1819,13 +1820,13 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J27" s="6">
         <v>-878424227</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L27" s="3">
         <v>2022</v>
@@ -1833,7 +1834,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>19</v>
@@ -1857,13 +1858,13 @@
         <v>50</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J28" s="6">
         <v>-4709453212</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L28" s="3">
         <v>2024</v>
@@ -1871,7 +1872,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>10</v>
@@ -1895,13 +1896,13 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J29" s="6">
         <v>-4906367157</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L29" s="3">
         <v>2026</v>
@@ -1909,7 +1910,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>10</v>
@@ -1933,13 +1934,13 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J30" s="6">
         <v>-942218135</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L30" s="3">
         <v>2023</v>
@@ -1947,7 +1948,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>10</v>
@@ -1971,13 +1972,13 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J31" s="6">
         <v>-4073830216</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L31" s="3">
         <v>2024</v>
@@ -1985,7 +1986,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>10</v>
@@ -2009,13 +2010,13 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J32" s="6">
         <v>-1002573664656</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L32" s="3">
         <v>2024</v>
@@ -2023,7 +2024,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>10</v>
@@ -2047,13 +2048,13 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J33" s="6">
         <v>-5079133035</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L33" s="3">
         <v>2026</v>
@@ -2061,7 +2062,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>19</v>
@@ -2085,13 +2086,13 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J34" s="6">
         <v>-4542263709</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L34" s="3">
         <v>2025</v>
@@ -2099,7 +2100,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>10</v>
@@ -2123,13 +2124,13 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J35" s="6">
         <v>-4102964588</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L35" s="3">
         <v>2024</v>
@@ -2137,7 +2138,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>10</v>
@@ -2161,13 +2162,13 @@
         <v>100</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J36" s="6">
         <v>-4092316930</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L36" s="3">
         <v>2024</v>
@@ -2175,7 +2176,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>10</v>
@@ -2199,13 +2200,13 @@
         <v>100</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J37" s="6">
         <v>-4891752359</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L37" s="3">
         <v>2026</v>
@@ -2213,7 +2214,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>10</v>
@@ -2237,13 +2238,13 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J38" s="6">
         <v>-892164059</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L38" s="3">
         <v>2023</v>
@@ -2251,7 +2252,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>10</v>
@@ -2275,13 +2276,13 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J39" s="6">
         <v>-1002035879507</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L39" s="3">
         <v>2022</v>
@@ -2289,7 +2290,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>19</v>
@@ -2313,13 +2314,13 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J40" s="6">
         <v>-4980553625</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L40" s="3">
         <v>2026</v>
@@ -2327,7 +2328,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>10</v>
@@ -2351,13 +2352,13 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J41" s="6">
         <v>-4875829621</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L41" s="3">
         <v>2026</v>
@@ -2365,7 +2366,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>10</v>
@@ -2389,13 +2390,13 @@
         <v>100</v>
       </c>
       <c r="I42" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J42" s="6">
         <v>-1002070587931</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L42" s="3">
         <v>2021</v>
@@ -2403,7 +2404,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>10</v>
@@ -2427,13 +2428,13 @@
         <v>100</v>
       </c>
       <c r="I43" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J43" s="6">
         <v>-889355707</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L43" s="3">
         <v>2021</v>
@@ -2441,7 +2442,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>10</v>
@@ -2465,13 +2466,13 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J44" s="6">
         <v>-4602706028</v>
       </c>
       <c r="K44" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L44" s="3">
         <v>2025</v>
@@ -2479,7 +2480,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>10</v>
@@ -2503,13 +2504,13 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J45" s="6">
         <v>-824212567</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L45" s="3">
         <v>2023</v>
@@ -2517,7 +2518,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>10</v>
@@ -2541,13 +2542,13 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J46" s="6">
         <v>-4595042190</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L46" s="3">
         <v>2025</v>
@@ -2555,7 +2556,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>10</v>
@@ -2579,13 +2580,13 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J47" s="6">
         <v>-1002012887954</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L47" s="3">
         <v>2021</v>
@@ -2593,7 +2594,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>19</v>
@@ -2617,13 +2618,13 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J48" s="6">
         <v>-4997646337</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L48" s="3">
         <v>2022</v>

</xml_diff>